<commit_message>
Verify platform eligibility for India-based orthopaedic surgeon; rebuild tracker
DataAnnotation (US/CA/UK/IE/AU/NZ only) and Handshake AI (US-only)
removed; Mercor corrected to the International Physicians track with
US/Canada-only specialist rates flagged; Meridial and Alignerr confirmed
India-eligible; specialty-demand caveat documented; tracker priorities
re-ordered accordingly and C8 platform row uncertainty noted.

Co-Authored-By: Claude <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01E1aigp4wPwpMwqvobhbDv6
</commit_message>
<xml_diff>
--- a/orthoos-v2/OrthoOS-side-income-tracker.xlsx
+++ b/orthoos-v2/OrthoOS-side-income-tracker.xlsx
@@ -719,30 +719,30 @@
       </c>
       <c r="B2" s="7" t="inlineStr">
         <is>
-          <t>Physician Talent Network</t>
+          <t>Healthcare Expert - INTERNATIONAL Physicians track</t>
         </is>
       </c>
       <c r="C2" s="7" t="inlineStr">
         <is>
-          <t>work.mercor.com</t>
+          <t>work.mercor.com (search: Healthcare Expert - International Physicians)</t>
         </is>
       </c>
       <c r="D2" s="7" t="inlineStr">
         <is>
-          <t>Yes (pays via Stripe)</t>
+          <t>YES (verified): MBBS accepted; dedicated international-physician posting; pays India via Stripe</t>
         </is>
       </c>
       <c r="E2" s="7" t="inlineStr">
         <is>
-          <t>100-210 (MD); specialty higher</t>
+          <t>50-180 healthcare band; $130-400 rates are US/Canada-practising tracks</t>
         </is>
       </c>
       <c r="F2" s="7">
-        <f>'Read Me'!$B$17*100</f>
+        <f>'Read Me'!$B$17*50</f>
         <v/>
       </c>
       <c r="G2" s="7">
-        <f>'Read Me'!$B$17*210</f>
+        <f>'Read Me'!$B$17*180</f>
         <v/>
       </c>
       <c r="H2" s="7" t="n">
@@ -756,7 +756,7 @@
       <c r="J2" s="8" t="inlineStr"/>
       <c r="K2" s="8" t="inlineStr">
         <is>
-          <t>3-stage: profile, written sample, 15-min AI video interview (3 attempts)</t>
+          <t>3-stage: profile, written sample, 15-min AI video interview (3 attempts); active licence + 5y experience</t>
         </is>
       </c>
       <c r="L2" s="8" t="inlineStr"/>
@@ -772,38 +772,38 @@
       </c>
       <c r="P2" s="8" t="inlineStr">
         <is>
-          <t>Top payer for physicians; lead profile with credential line</t>
+          <t>VERIFIED: specialist roles (cardiology etc. $180-400) require US/Canada practice. Apply to the International Physicians track and confirm ITS rate before committing hours</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="7" t="inlineStr">
         <is>
-          <t>Handshake AI</t>
+          <t>Invisible Tech (Meridial)</t>
         </is>
       </c>
       <c r="B3" s="7" t="inlineStr">
         <is>
-          <t>AI tutor / expert (postgrad)</t>
+          <t>Domain expert - healthcare</t>
         </is>
       </c>
       <c r="C3" s="7" t="inlineStr">
         <is>
-          <t>joinhandshake.com / edtech listing</t>
+          <t>meridial.ai/projects</t>
         </is>
       </c>
       <c r="D3" s="7" t="inlineStr">
         <is>
-          <t>Verify per posting</t>
+          <t>YES (verified): India in eligible regions (US/CA/UK/EU/MX/BR/IN/JP/KR/SG)</t>
         </is>
       </c>
       <c r="E3" s="7" t="inlineStr">
         <is>
-          <t>up to 125</t>
+          <t>35-125 domain experts</t>
         </is>
       </c>
       <c r="F3" s="7">
-        <f>'Read Me'!$B$17*60</f>
+        <f>'Read Me'!$B$17*35</f>
         <v/>
       </c>
       <c r="G3" s="7">
@@ -819,7 +819,11 @@
         </is>
       </c>
       <c r="J3" s="8" t="inlineStr"/>
-      <c r="K3" s="8" t="inlineStr"/>
+      <c r="K3" s="8" t="inlineStr">
+        <is>
+          <t>Apply at meridial.ai; invitations reviewed ~48h</t>
+        </is>
+      </c>
       <c r="L3" s="8" t="inlineStr"/>
       <c r="M3" s="8" t="inlineStr"/>
       <c r="N3" s="7">
@@ -833,42 +837,42 @@
       </c>
       <c r="P3" s="8" t="inlineStr">
         <is>
-          <t>Targets MS/PhD/postdoc; statistics training qualifies</t>
+          <t>One of only two platforms with India EXPLICITLY listed</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="7" t="inlineStr">
         <is>
-          <t>Outlier (Scale AI)</t>
+          <t>Alignerr (Labelbox)</t>
         </is>
       </c>
       <c r="B4" s="7" t="inlineStr">
         <is>
-          <t>Radiology / medical expert</t>
+          <t>Medical expert</t>
         </is>
       </c>
       <c r="C4" s="7" t="inlineStr">
         <is>
-          <t>outlier.ai/experts/radiology</t>
+          <t>alignerr.com</t>
         </is>
       </c>
       <c r="D4" s="7" t="inlineStr">
         <is>
-          <t>Verify per posting</t>
+          <t>YES (verified): India in published 14-country eligibility set</t>
         </is>
       </c>
       <c r="E4" s="7" t="inlineStr">
         <is>
-          <t>up to 150 specialty; 15-50 generalist</t>
+          <t>30-100 (varies by project)</t>
         </is>
       </c>
       <c r="F4" s="7">
-        <f>'Read Me'!$B$17*40</f>
+        <f>'Read Me'!$B$17*30</f>
         <v/>
       </c>
       <c r="G4" s="7">
-        <f>'Read Me'!$B$17*150</f>
+        <f>'Read Me'!$B$17*100</f>
         <v/>
       </c>
       <c r="H4" s="7" t="n">
@@ -894,46 +898,46 @@
       </c>
       <c r="P4" s="8" t="inlineStr">
         <is>
-          <t>Only specialty tracks clear the Rs 4k/h floor</t>
+          <t>India explicitly eligible</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="7" t="inlineStr">
         <is>
-          <t>DataAnnotation</t>
+          <t>OpenTrain (aggregator)</t>
         </is>
       </c>
       <c r="B5" s="7" t="inlineStr">
         <is>
-          <t>Medicine track</t>
+          <t>Profile + job alerts</t>
         </is>
       </c>
       <c r="C5" s="7" t="inlineStr">
         <is>
-          <t>dataannotation.tech/medicine</t>
+          <t>opentrain.ai</t>
         </is>
       </c>
       <c r="D5" s="7" t="inlineStr">
         <is>
-          <t>Verify</t>
+          <t>Aggregator - eligibility is per posting</t>
         </is>
       </c>
       <c r="E5" s="7" t="inlineStr">
         <is>
-          <t>40-50+ medical</t>
+          <t>25-100 clinical postings</t>
         </is>
       </c>
       <c r="F5" s="7">
-        <f>'Read Me'!$B$17*40</f>
+        <f>'Read Me'!$B$17*25</f>
         <v/>
       </c>
       <c r="G5" s="7">
-        <f>'Read Me'!$B$17*60</f>
+        <f>'Read Me'!$B$17*100</f>
         <v/>
       </c>
       <c r="H5" s="7" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="I5" s="8" t="inlineStr">
         <is>
@@ -950,47 +954,47 @@
       </c>
       <c r="O5" s="8" t="inlineStr">
         <is>
-          <t>Apply Day 2</t>
+          <t>Create profile Day 1</t>
         </is>
       </c>
       <c r="P5" s="8" t="inlineStr">
         <is>
-          <t>Steadier volume, lower ceiling</t>
+          <t>Weekly Monday scan; filter India-eligible postings</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="7" t="inlineStr">
         <is>
-          <t>Turing</t>
+          <t>Outlier (Scale AI)</t>
         </is>
       </c>
       <c r="B6" s="7" t="inlineStr">
         <is>
-          <t>Medical SME</t>
+          <t>Medical/generalist (radiology track likely US-focused)</t>
         </is>
       </c>
       <c r="C6" s="7" t="inlineStr">
         <is>
-          <t>turing.com</t>
+          <t>outlier.ai</t>
         </is>
       </c>
       <c r="D6" s="7" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>PARTIAL (verified): India live (~50 countries) BUT task volume prioritised US/UK/DE; VPN = instant ban</t>
         </is>
       </c>
       <c r="E6" s="7" t="inlineStr">
         <is>
-          <t>varies by project</t>
+          <t>15-50 generalist; specialty higher where offered</t>
         </is>
       </c>
       <c r="F6" s="7">
-        <f>'Read Me'!$B$17*30</f>
+        <f>'Read Me'!$B$17*15</f>
         <v/>
       </c>
       <c r="G6" s="7">
-        <f>'Read Me'!$B$17*100</f>
+        <f>'Read Me'!$B$17*50</f>
         <v/>
       </c>
       <c r="H6" s="7" t="n">
@@ -1002,7 +1006,11 @@
         </is>
       </c>
       <c r="J6" s="8" t="inlineStr"/>
-      <c r="K6" s="8" t="inlineStr"/>
+      <c r="K6" s="8" t="inlineStr">
+        <is>
+          <t>ID + location verification at onboarding</t>
+        </is>
+      </c>
       <c r="L6" s="8" t="inlineStr"/>
       <c r="M6" s="8" t="inlineStr"/>
       <c r="N6" s="7">
@@ -1014,40 +1022,44 @@
           <t>Apply Day 2</t>
         </is>
       </c>
-      <c r="P6" s="8" t="inlineStr"/>
+      <c r="P6" s="8" t="inlineStr">
+        <is>
+          <t>Expect thin task flow from India; keep only if effective rate clears Rs 4k/h</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="7" t="inlineStr">
         <is>
-          <t>Alignerr (Labelbox)</t>
+          <t>Micro1</t>
         </is>
       </c>
       <c r="B7" s="7" t="inlineStr">
         <is>
-          <t>Medical expert</t>
+          <t>Medical expert / evaluator</t>
         </is>
       </c>
       <c r="C7" s="7" t="inlineStr">
         <is>
-          <t>alignerr.com</t>
+          <t>micro1.ai/experts</t>
         </is>
       </c>
       <c r="D7" s="7" t="inlineStr">
         <is>
-          <t>Verify</t>
+          <t>LIKELY: healthcare domain listed, medical-expert postings live; country set not published</t>
         </is>
       </c>
       <c r="E7" s="7" t="inlineStr">
         <is>
-          <t>varies</t>
+          <t>20-65 evaluator</t>
         </is>
       </c>
       <c r="F7" s="7">
-        <f>'Read Me'!$B$17*30</f>
+        <f>'Read Me'!$B$17*20</f>
         <v/>
       </c>
       <c r="G7" s="7">
-        <f>'Read Me'!$B$17*100</f>
+        <f>'Read Me'!$B$17*65</f>
         <v/>
       </c>
       <c r="H7" s="7" t="n">
@@ -1071,32 +1083,36 @@
           <t>Apply Day 2</t>
         </is>
       </c>
-      <c r="P7" s="8" t="inlineStr"/>
+      <c r="P7" s="8" t="inlineStr">
+        <is>
+          <t>Physician feedback reports wide/lower variance</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="7" t="inlineStr">
         <is>
-          <t>Micro1</t>
+          <t>Toloka / Mindrift</t>
         </is>
       </c>
       <c r="B8" s="7" t="inlineStr">
         <is>
-          <t>Evaluator</t>
+          <t>Medicine domain</t>
         </is>
       </c>
       <c r="C8" s="7" t="inlineStr">
         <is>
-          <t>micro1.ai</t>
+          <t>mindrift.ai</t>
         </is>
       </c>
       <c r="D8" s="7" t="inlineStr">
         <is>
-          <t>Verify</t>
+          <t>YES (verified): join from any country</t>
         </is>
       </c>
       <c r="E8" s="7" t="inlineStr">
         <is>
-          <t>20-65 evaluator</t>
+          <t>20-60</t>
         </is>
       </c>
       <c r="F8" s="7">
@@ -1104,7 +1120,7 @@
         <v/>
       </c>
       <c r="G8" s="7">
-        <f>'Read Me'!$B$17*65</f>
+        <f>'Read Me'!$B$17*60</f>
         <v/>
       </c>
       <c r="H8" s="7" t="n">
@@ -1125,47 +1141,47 @@
       </c>
       <c r="O8" s="8" t="inlineStr">
         <is>
-          <t>Apply Day 3</t>
+          <t>Apply Day 2</t>
         </is>
       </c>
       <c r="P8" s="8" t="inlineStr">
         <is>
-          <t>Physician feedback reports wide/lower variance</t>
+          <t>Lower rates - volume filler only if above Rs 4k/h</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="7" t="inlineStr">
         <is>
-          <t>Pareto AI</t>
+          <t>Turing</t>
         </is>
       </c>
       <c r="B9" s="7" t="inlineStr">
         <is>
-          <t>AI trainer</t>
+          <t>Medical SME</t>
         </is>
       </c>
       <c r="C9" s="7" t="inlineStr">
         <is>
-          <t>pareto.ai</t>
+          <t>turing.com</t>
         </is>
       </c>
       <c r="D9" s="7" t="inlineStr">
         <is>
-          <t>Verify</t>
+          <t>UNVERIFIED for medical roles - check current postings</t>
         </is>
       </c>
       <c r="E9" s="7" t="inlineStr">
         <is>
-          <t>35-60 reported</t>
+          <t>varies by project</t>
         </is>
       </c>
       <c r="F9" s="7">
-        <f>'Read Me'!$B$17*35</f>
+        <f>'Read Me'!$B$17*30</f>
         <v/>
       </c>
       <c r="G9" s="7">
-        <f>'Read Me'!$B$17*60</f>
+        <f>'Read Me'!$B$17*100</f>
         <v/>
       </c>
       <c r="H9" s="7" t="n">
@@ -1191,46 +1207,46 @@
       </c>
       <c r="P9" s="8" t="inlineStr">
         <is>
-          <t>Rates not published</t>
+          <t>No India-specific medical evidence found in research</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="7" t="inlineStr">
         <is>
-          <t>Invisible Technologies</t>
+          <t>Pareto AI</t>
         </is>
       </c>
       <c r="B10" s="7" t="inlineStr">
         <is>
-          <t>Expert marketplace</t>
+          <t>AI trainer</t>
         </is>
       </c>
       <c r="C10" s="7" t="inlineStr">
         <is>
-          <t>invisible.co</t>
+          <t>pareto.ai</t>
         </is>
       </c>
       <c r="D10" s="7" t="inlineStr">
         <is>
-          <t>Verify</t>
+          <t>UNVERIFIED - rates and countries not published</t>
         </is>
       </c>
       <c r="E10" s="7" t="inlineStr">
         <is>
-          <t>varies</t>
+          <t>35-60 reported</t>
         </is>
       </c>
       <c r="F10" s="7">
-        <f>'Read Me'!$B$17*25</f>
+        <f>'Read Me'!$B$17*35</f>
         <v/>
       </c>
       <c r="G10" s="7">
-        <f>'Read Me'!$B$17*80</f>
+        <f>'Read Me'!$B$17*60</f>
         <v/>
       </c>
       <c r="H10" s="7" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="I10" s="8" t="inlineStr">
         <is>
@@ -1247,7 +1263,7 @@
       </c>
       <c r="O10" s="8" t="inlineStr">
         <is>
-          <t>Apply Day 3</t>
+          <t>Apply Day 3 if time</t>
         </is>
       </c>
       <c r="P10" s="8" t="inlineStr"/>
@@ -1255,7 +1271,7 @@
     <row r="11">
       <c r="A11" s="7" t="inlineStr">
         <is>
-          <t>Toloka / Mindrift</t>
+          <t>Sepal AI</t>
         </is>
       </c>
       <c r="B11" s="7" t="inlineStr">
@@ -1265,25 +1281,25 @@
       </c>
       <c r="C11" s="7" t="inlineStr">
         <is>
-          <t>mindrift.ai</t>
+          <t>sepal.ai</t>
         </is>
       </c>
       <c r="D11" s="7" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>UNVERIFIED - nothing found in research</t>
         </is>
       </c>
       <c r="E11" s="7" t="inlineStr">
         <is>
-          <t>20-60</t>
+          <t>unknown</t>
         </is>
       </c>
       <c r="F11" s="7">
-        <f>'Read Me'!$B$17*20</f>
+        <f>'Read Me'!$B$17*25</f>
         <v/>
       </c>
       <c r="G11" s="7">
-        <f>'Read Me'!$B$17*60</f>
+        <f>'Read Me'!$B$17*80</f>
         <v/>
       </c>
       <c r="H11" s="7" t="n">
@@ -1304,7 +1320,7 @@
       </c>
       <c r="O11" s="8" t="inlineStr">
         <is>
-          <t>Apply Day 3</t>
+          <t>Skip unless posting found</t>
         </is>
       </c>
       <c r="P11" s="8" t="inlineStr"/>
@@ -1312,35 +1328,35 @@
     <row r="12">
       <c r="A12" s="7" t="inlineStr">
         <is>
-          <t>Sepal AI</t>
+          <t>Centific</t>
         </is>
       </c>
       <c r="B12" s="7" t="inlineStr">
         <is>
-          <t>Medical expert</t>
+          <t>Healthcare data</t>
         </is>
       </c>
       <c r="C12" s="7" t="inlineStr">
         <is>
-          <t>sepal.ai</t>
+          <t>centific.com</t>
         </is>
       </c>
       <c r="D12" s="7" t="inlineStr">
         <is>
-          <t>Verify</t>
+          <t>UNVERIFIED</t>
         </is>
       </c>
       <c r="E12" s="7" t="inlineStr">
         <is>
-          <t>varies</t>
+          <t>unknown</t>
         </is>
       </c>
       <c r="F12" s="7">
-        <f>'Read Me'!$B$17*25</f>
+        <f>'Read Me'!$B$17*20</f>
         <v/>
       </c>
       <c r="G12" s="7">
-        <f>'Read Me'!$B$17*80</f>
+        <f>'Read Me'!$B$17*60</f>
         <v/>
       </c>
       <c r="H12" s="7" t="n">
@@ -1361,7 +1377,7 @@
       </c>
       <c r="O12" s="8" t="inlineStr">
         <is>
-          <t>Apply Day 3</t>
+          <t>Skip unless posting found</t>
         </is>
       </c>
       <c r="P12" s="8" t="inlineStr"/>
@@ -1369,43 +1385,43 @@
     <row r="13">
       <c r="A13" s="7" t="inlineStr">
         <is>
-          <t>Centific</t>
+          <t>DataAnnotation</t>
         </is>
       </c>
       <c r="B13" s="7" t="inlineStr">
         <is>
-          <t>Healthcare data</t>
+          <t>Medicine track</t>
         </is>
       </c>
       <c r="C13" s="7" t="inlineStr">
         <is>
-          <t>centific.com</t>
+          <t>dataannotation.tech</t>
         </is>
       </c>
       <c r="D13" s="7" t="inlineStr">
         <is>
-          <t>Verify</t>
+          <t>NO (verified): US/CA/UK/IE/AU/NZ only</t>
         </is>
       </c>
       <c r="E13" s="7" t="inlineStr">
         <is>
-          <t>varies</t>
+          <t>40-50+ medical (not accessible from India)</t>
         </is>
       </c>
       <c r="F13" s="7">
-        <f>'Read Me'!$B$17*20</f>
+        <f>'Read Me'!$B$17*0</f>
         <v/>
       </c>
       <c r="G13" s="7">
-        <f>'Read Me'!$B$17*60</f>
+        <f>'Read Me'!$B$17*0</f>
         <v/>
       </c>
       <c r="H13" s="7" t="n">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="I13" s="8" t="inlineStr">
         <is>
-          <t>Not applied</t>
+          <t>NOT ELIGIBLE</t>
         </is>
       </c>
       <c r="J13" s="8" t="inlineStr"/>
@@ -1418,51 +1434,55 @@
       </c>
       <c r="O13" s="8" t="inlineStr">
         <is>
-          <t>Apply Day 3</t>
-        </is>
-      </c>
-      <c r="P13" s="8" t="inlineStr"/>
+          <t>Skip</t>
+        </is>
+      </c>
+      <c r="P13" s="8" t="inlineStr">
+        <is>
+          <t>Removed from plan - India not in eligibility set</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="7" t="inlineStr">
         <is>
-          <t>OpenTrain (aggregator)</t>
+          <t>Handshake AI</t>
         </is>
       </c>
       <c r="B14" s="7" t="inlineStr">
         <is>
-          <t>Profile + job alerts</t>
+          <t>AI tutor / fellowship</t>
         </is>
       </c>
       <c r="C14" s="7" t="inlineStr">
         <is>
-          <t>opentrain.ai</t>
+          <t>joinhandshake.com/ai</t>
         </is>
       </c>
       <c r="D14" s="7" t="inlineStr">
         <is>
-          <t>Aggregator</t>
+          <t>NO (verified): US-based with US work authorisation only</t>
         </is>
       </c>
       <c r="E14" s="7" t="inlineStr">
         <is>
-          <t>25-100 clinical postings</t>
+          <t>up to 125 (not accessible from India)</t>
         </is>
       </c>
       <c r="F14" s="7">
-        <f>'Read Me'!$B$17*25</f>
+        <f>'Read Me'!$B$17*0</f>
         <v/>
       </c>
       <c r="G14" s="7">
-        <f>'Read Me'!$B$17*100</f>
+        <f>'Read Me'!$B$17*0</f>
         <v/>
       </c>
       <c r="H14" s="7" t="n">
-        <v>2</v>
+        <v>9</v>
       </c>
       <c r="I14" s="8" t="inlineStr">
         <is>
-          <t>Not applied</t>
+          <t>NOT ELIGIBLE</t>
         </is>
       </c>
       <c r="J14" s="8" t="inlineStr"/>
@@ -1475,12 +1495,12 @@
       </c>
       <c r="O14" s="8" t="inlineStr">
         <is>
-          <t>Create profile Day 1</t>
+          <t>Skip</t>
         </is>
       </c>
       <c r="P14" s="8" t="inlineStr">
         <is>
-          <t>Use for weekly Monday scan</t>
+          <t>Removed from plan - US-only program</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Verify outreach recipient addresses; update tracker with confirmed routes
partner@qure.ai, info@imagebiopsy.com, partner@lunit.io corrected from
guesses; DeepTek/Gleamer/Radiobotics/Aidoc guesses confirmed; AZmed has
no public general address (named contact + web form); Annalise.ai is
web-form only. Gmail draft To: fields updated to match.

Co-Authored-By: Claude <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01E1aigp4wPwpMwqvobhbDv6
</commit_message>
<xml_diff>
--- a/orthoos-v2/OrthoOS-side-income-tracker.xlsx
+++ b/orthoos-v2/OrthoOS-side-income-tracker.xlsx
@@ -1618,7 +1618,7 @@
       </c>
       <c r="C2" s="7" t="inlineStr">
         <is>
-          <t>Mumbai, India</t>
+          <t>Mumbai, India / NYC</t>
         </is>
       </c>
       <c r="D2" s="7" t="inlineStr">
@@ -1628,7 +1628,7 @@
       </c>
       <c r="E2" s="7" t="inlineStr">
         <is>
-          <t>Indian; easiest first meeting; MSK product line</t>
+          <t>Indian roots; MSK product line; note: no ortho job openings - this is a VENDOR pitch, not an application</t>
         </is>
       </c>
       <c r="F2" s="7" t="inlineStr">
@@ -1638,12 +1638,12 @@
       </c>
       <c r="G2" s="8" t="inlineStr">
         <is>
-          <t>partnerships@qure.ai</t>
+          <t>partner@qure.ai (VERIFIED - partnerships address; careers@qure.ai exists separately)</t>
         </is>
       </c>
       <c r="H2" s="7" t="inlineStr">
         <is>
-          <t>Draft ready</t>
+          <t>Draft ready + addressed</t>
         </is>
       </c>
       <c r="I2" s="8" t="inlineStr">
@@ -1655,7 +1655,7 @@
       <c r="K2" s="8" t="inlineStr"/>
       <c r="L2" s="8" t="inlineStr">
         <is>
-          <t>Verify address on qure.ai contact page</t>
+          <t>Send wave 1</t>
         </is>
       </c>
       <c r="M2" s="8" t="inlineStr"/>
@@ -1686,17 +1686,17 @@
       </c>
       <c r="F3" s="7" t="inlineStr">
         <is>
-          <t>Email + LinkedIn</t>
+          <t>Email + LinkedIn + phone</t>
         </is>
       </c>
       <c r="G3" s="8" t="inlineStr">
         <is>
-          <t>info@deeptek.ai</t>
+          <t>info@deeptek.ai (VERIFIED, official site) | ph +91 96070 82012</t>
         </is>
       </c>
       <c r="H3" s="7" t="inlineStr">
         <is>
-          <t>Draft ready</t>
+          <t>Draft ready + addressed</t>
         </is>
       </c>
       <c r="I3" s="8" t="inlineStr">
@@ -1708,7 +1708,7 @@
       <c r="K3" s="8" t="inlineStr"/>
       <c r="L3" s="8" t="inlineStr">
         <is>
-          <t>Verify address on deeptek.ai</t>
+          <t>Send wave 1</t>
         </is>
       </c>
       <c r="M3" s="8" t="inlineStr"/>
@@ -1744,12 +1744,12 @@
       </c>
       <c r="G4" s="8" t="inlineStr">
         <is>
-          <t>office@imagebiopsy.com</t>
+          <t>info@imagebiopsy.com (VERIFIED, official contact page; support@ for existing customers)</t>
         </is>
       </c>
       <c r="H4" s="7" t="inlineStr">
         <is>
-          <t>Draft ready</t>
+          <t>Draft ready + addressed</t>
         </is>
       </c>
       <c r="I4" s="8" t="inlineStr">
@@ -1761,7 +1761,7 @@
       <c r="K4" s="8" t="inlineStr"/>
       <c r="L4" s="8" t="inlineStr">
         <is>
-          <t>Verify address on imagebiopsy.com</t>
+          <t>Send wave 1</t>
         </is>
       </c>
       <c r="M4" s="8" t="inlineStr"/>
@@ -1797,12 +1797,12 @@
       </c>
       <c r="G5" s="8" t="inlineStr">
         <is>
-          <t>contact@gleamer.ai</t>
+          <t>contact@gleamer.ai (VERIFIED via healthcare-in-europe directory)</t>
         </is>
       </c>
       <c r="H5" s="7" t="inlineStr">
         <is>
-          <t>Draft ready</t>
+          <t>Draft ready + addressed</t>
         </is>
       </c>
       <c r="I5" s="8" t="inlineStr">
@@ -1814,7 +1814,7 @@
       <c r="K5" s="8" t="inlineStr"/>
       <c r="L5" s="8" t="inlineStr">
         <is>
-          <t>Verify address on gleamer.ai</t>
+          <t>Send wave 2</t>
         </is>
       </c>
       <c r="M5" s="8" t="inlineStr"/>
@@ -1850,12 +1850,12 @@
       </c>
       <c r="G6" s="8" t="inlineStr">
         <is>
-          <t>info@radiobotics.com</t>
+          <t>info@radiobotics.com (VERIFIED via directory)</t>
         </is>
       </c>
       <c r="H6" s="7" t="inlineStr">
         <is>
-          <t>Draft ready</t>
+          <t>Draft ready + addressed</t>
         </is>
       </c>
       <c r="I6" s="8" t="inlineStr">
@@ -1867,7 +1867,7 @@
       <c r="K6" s="8" t="inlineStr"/>
       <c r="L6" s="8" t="inlineStr">
         <is>
-          <t>Verify address on radiobotics.com</t>
+          <t>Send wave 2</t>
         </is>
       </c>
       <c r="M6" s="8" t="inlineStr"/>
@@ -1893,22 +1893,22 @@
       </c>
       <c r="E7" s="7" t="inlineStr">
         <is>
-          <t>Competes on sensitivity claims -&gt; needs validation evidence</t>
+          <t>Sensitivity-led claims need validation evidence</t>
         </is>
       </c>
       <c r="F7" s="7" t="inlineStr">
         <is>
-          <t>Email + LinkedIn</t>
+          <t>Email + LinkedIn + web form</t>
         </is>
       </c>
       <c r="G7" s="8" t="inlineStr">
         <is>
-          <t>contact@azmed.co</t>
+          <t>anthony@azmed.co (directory-sourced named contact; no general address published - azmed.co/contact form is the official route)</t>
         </is>
       </c>
       <c r="H7" s="7" t="inlineStr">
         <is>
-          <t>Draft ready</t>
+          <t>Draft ready + addressed</t>
         </is>
       </c>
       <c r="I7" s="8" t="inlineStr">
@@ -1920,7 +1920,7 @@
       <c r="K7" s="8" t="inlineStr"/>
       <c r="L7" s="8" t="inlineStr">
         <is>
-          <t>Verify address on azmed.co</t>
+          <t>Send wave 2; expect possible bounce -&gt; use form</t>
         </is>
       </c>
       <c r="M7" s="8" t="inlineStr"/>
@@ -1956,12 +1956,12 @@
       </c>
       <c r="G8" s="8" t="inlineStr">
         <is>
-          <t>contact@lunit.io</t>
+          <t>partner@lunit.io (VERIFIED, official contact page; also contact@lunit.io)</t>
         </is>
       </c>
       <c r="H8" s="7" t="inlineStr">
         <is>
-          <t>Draft ready</t>
+          <t>Draft ready + addressed</t>
         </is>
       </c>
       <c r="I8" s="8" t="inlineStr">
@@ -1973,7 +1973,7 @@
       <c r="K8" s="8" t="inlineStr"/>
       <c r="L8" s="8" t="inlineStr">
         <is>
-          <t>Verify address on lunit.io</t>
+          <t>Send wave 2</t>
         </is>
       </c>
       <c r="M8" s="8" t="inlineStr"/>
@@ -1989,7 +1989,7 @@
       </c>
       <c r="C9" s="7" t="inlineStr">
         <is>
-          <t>Tel Aviv, Israel</t>
+          <t>Tel Aviv / NYC</t>
         </is>
       </c>
       <c r="D9" s="7" t="inlineStr">
@@ -2009,12 +2009,12 @@
       </c>
       <c r="G9" s="8" t="inlineStr">
         <is>
-          <t>info@aidoc.com</t>
+          <t>info@aidoc.com (VERIFIED via directory)</t>
         </is>
       </c>
       <c r="H9" s="7" t="inlineStr">
         <is>
-          <t>Draft ready</t>
+          <t>Draft ready + addressed</t>
         </is>
       </c>
       <c r="I9" s="8" t="inlineStr">
@@ -2026,7 +2026,7 @@
       <c r="K9" s="8" t="inlineStr"/>
       <c r="L9" s="8" t="inlineStr">
         <is>
-          <t>Verify address on aidoc.com</t>
+          <t>Send wave 3</t>
         </is>
       </c>
       <c r="M9" s="8" t="inlineStr"/>
@@ -2037,7 +2037,7 @@
       </c>
       <c r="B10" s="7" t="inlineStr">
         <is>
-          <t>Annalise.ai</t>
+          <t>Annalise.ai (harrison.ai)</t>
         </is>
       </c>
       <c r="C10" s="7" t="inlineStr">
@@ -2057,17 +2057,17 @@
       </c>
       <c r="F10" s="7" t="inlineStr">
         <is>
-          <t>Email + LinkedIn</t>
+          <t>WEB FORM (no public email; staff use @harrison.ai)</t>
         </is>
       </c>
       <c r="G10" s="8" t="inlineStr">
         <is>
-          <t>info@annalise.ai</t>
+          <t>NO EMAIL - use usa.annalise.ai/contact/general-enquiry; paste draft text</t>
         </is>
       </c>
       <c r="H10" s="7" t="inlineStr">
         <is>
-          <t>Draft ready</t>
+          <t>Draft text ready (paste into form)</t>
         </is>
       </c>
       <c r="I10" s="8" t="inlineStr">
@@ -2079,7 +2079,7 @@
       <c r="K10" s="8" t="inlineStr"/>
       <c r="L10" s="8" t="inlineStr">
         <is>
-          <t>Verify address on annalise.ai</t>
+          <t>Submit via form, wave 3</t>
         </is>
       </c>
       <c r="M10" s="8" t="inlineStr"/>
@@ -2105,7 +2105,7 @@
       </c>
       <c r="E11" s="7" t="inlineStr">
         <is>
-          <t>HealthBench-style physician rubric programs; route via Mercor/Handshake postings + direct careers pages</t>
+          <t>HealthBench-style physician rubric programs</t>
         </is>
       </c>
       <c r="F11" s="7" t="inlineStr">
@@ -2113,10 +2113,14 @@
           <t>Careers pages + platform postings</t>
         </is>
       </c>
-      <c r="G11" s="8" t="inlineStr"/>
+      <c r="G11" s="8" t="inlineStr">
+        <is>
+          <t>N/A - apply via portal</t>
+        </is>
+      </c>
       <c r="H11" s="7" t="inlineStr">
         <is>
-          <t>N/A - apply via portal</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="I11" s="8" t="inlineStr">

</xml_diff>

<commit_message>
Mark 8 outreach emails as sent in tracker
Co-Authored-By: Claude <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01E1aigp4wPwpMwqvobhbDv6
</commit_message>
<xml_diff>
--- a/orthoos-v2/OrthoOS-side-income-tracker.xlsx
+++ b/orthoos-v2/OrthoOS-side-income-tracker.xlsx
@@ -1643,19 +1643,19 @@
       </c>
       <c r="H2" s="7" t="inlineStr">
         <is>
-          <t>Draft ready + addressed</t>
+          <t>SENT</t>
         </is>
       </c>
       <c r="I2" s="8" t="inlineStr">
         <is>
-          <t>Not sent</t>
+          <t>Sent 20-Aug-2026</t>
         </is>
       </c>
       <c r="J2" s="8" t="inlineStr"/>
       <c r="K2" s="8" t="inlineStr"/>
       <c r="L2" s="8" t="inlineStr">
         <is>
-          <t>Send wave 1</t>
+          <t>Await reply; follow up in 7-10 days if none</t>
         </is>
       </c>
       <c r="M2" s="8" t="inlineStr"/>
@@ -1696,19 +1696,19 @@
       </c>
       <c r="H3" s="7" t="inlineStr">
         <is>
-          <t>Draft ready + addressed</t>
+          <t>SENT</t>
         </is>
       </c>
       <c r="I3" s="8" t="inlineStr">
         <is>
-          <t>Not sent</t>
+          <t>Sent 20-Aug-2026</t>
         </is>
       </c>
       <c r="J3" s="8" t="inlineStr"/>
       <c r="K3" s="8" t="inlineStr"/>
       <c r="L3" s="8" t="inlineStr">
         <is>
-          <t>Send wave 1</t>
+          <t>Await reply; follow up in 7-10 days if none</t>
         </is>
       </c>
       <c r="M3" s="8" t="inlineStr"/>
@@ -1749,19 +1749,19 @@
       </c>
       <c r="H4" s="7" t="inlineStr">
         <is>
-          <t>Draft ready + addressed</t>
+          <t>SENT</t>
         </is>
       </c>
       <c r="I4" s="8" t="inlineStr">
         <is>
-          <t>Not sent</t>
+          <t>Sent 20-Aug-2026</t>
         </is>
       </c>
       <c r="J4" s="8" t="inlineStr"/>
       <c r="K4" s="8" t="inlineStr"/>
       <c r="L4" s="8" t="inlineStr">
         <is>
-          <t>Send wave 1</t>
+          <t>Await reply; follow up in 7-10 days if none</t>
         </is>
       </c>
       <c r="M4" s="8" t="inlineStr"/>
@@ -1802,19 +1802,19 @@
       </c>
       <c r="H5" s="7" t="inlineStr">
         <is>
-          <t>Draft ready + addressed</t>
+          <t>SENT</t>
         </is>
       </c>
       <c r="I5" s="8" t="inlineStr">
         <is>
-          <t>Not sent</t>
+          <t>Sent 20-Aug-2026</t>
         </is>
       </c>
       <c r="J5" s="8" t="inlineStr"/>
       <c r="K5" s="8" t="inlineStr"/>
       <c r="L5" s="8" t="inlineStr">
         <is>
-          <t>Send wave 2</t>
+          <t>Await reply; follow up in 7-10 days if none</t>
         </is>
       </c>
       <c r="M5" s="8" t="inlineStr"/>
@@ -1855,19 +1855,19 @@
       </c>
       <c r="H6" s="7" t="inlineStr">
         <is>
-          <t>Draft ready + addressed</t>
+          <t>SENT</t>
         </is>
       </c>
       <c r="I6" s="8" t="inlineStr">
         <is>
-          <t>Not sent</t>
+          <t>Sent 20-Aug-2026</t>
         </is>
       </c>
       <c r="J6" s="8" t="inlineStr"/>
       <c r="K6" s="8" t="inlineStr"/>
       <c r="L6" s="8" t="inlineStr">
         <is>
-          <t>Send wave 2</t>
+          <t>Await reply; follow up in 7-10 days if none</t>
         </is>
       </c>
       <c r="M6" s="8" t="inlineStr"/>
@@ -1908,19 +1908,19 @@
       </c>
       <c r="H7" s="7" t="inlineStr">
         <is>
-          <t>Draft ready + addressed</t>
+          <t>SENT</t>
         </is>
       </c>
       <c r="I7" s="8" t="inlineStr">
         <is>
-          <t>Not sent</t>
+          <t>Sent 20-Aug-2026</t>
         </is>
       </c>
       <c r="J7" s="8" t="inlineStr"/>
       <c r="K7" s="8" t="inlineStr"/>
       <c r="L7" s="8" t="inlineStr">
         <is>
-          <t>Send wave 2; expect possible bounce -&gt; use form</t>
+          <t>Watch for bounce -&gt; if bounced, submit via azmed.co/contact form</t>
         </is>
       </c>
       <c r="M7" s="8" t="inlineStr"/>
@@ -1961,19 +1961,19 @@
       </c>
       <c r="H8" s="7" t="inlineStr">
         <is>
-          <t>Draft ready + addressed</t>
+          <t>SENT</t>
         </is>
       </c>
       <c r="I8" s="8" t="inlineStr">
         <is>
-          <t>Not sent</t>
+          <t>Sent 20-Aug-2026</t>
         </is>
       </c>
       <c r="J8" s="8" t="inlineStr"/>
       <c r="K8" s="8" t="inlineStr"/>
       <c r="L8" s="8" t="inlineStr">
         <is>
-          <t>Send wave 2</t>
+          <t>Await reply; follow up in 7-10 days if none</t>
         </is>
       </c>
       <c r="M8" s="8" t="inlineStr"/>
@@ -2014,19 +2014,19 @@
       </c>
       <c r="H9" s="7" t="inlineStr">
         <is>
-          <t>Draft ready + addressed</t>
+          <t>SENT</t>
         </is>
       </c>
       <c r="I9" s="8" t="inlineStr">
         <is>
-          <t>Not sent</t>
+          <t>Sent 20-Aug-2026</t>
         </is>
       </c>
       <c r="J9" s="8" t="inlineStr"/>
       <c r="K9" s="8" t="inlineStr"/>
       <c r="L9" s="8" t="inlineStr">
         <is>
-          <t>Send wave 3</t>
+          <t>Await reply; follow up in 7-10 days if none</t>
         </is>
       </c>
       <c r="M9" s="8" t="inlineStr"/>

</xml_diff>